<commit_message>
Implement tool acquisition and economy updates
</commit_message>
<xml_diff>
--- a/spec/Docs/01_Design/CardDesignVersion/物品列表.xlsx
+++ b/spec/Docs/01_Design/CardDesignVersion/物品列表.xlsx
@@ -3139,7 +3139,7 @@
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <dimension ref="A1:I16"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
@@ -3193,7 +3193,7 @@
         <v>11</v>
       </c>
       <c r="D2" s="2">
-        <v>18</v>
+        <v>5</v>
       </c>
       <c r="E2" s="2">
         <v>1</v>
@@ -3222,7 +3222,7 @@
         <v>11</v>
       </c>
       <c r="D3" s="2">
-        <v>20</v>
+        <v>6</v>
       </c>
       <c r="E3" s="2">
         <v>1</v>
@@ -3251,7 +3251,7 @@
         <v>11</v>
       </c>
       <c r="D4" s="2">
-        <v>22</v>
+        <v>6</v>
       </c>
       <c r="E4" s="2">
         <v>1</v>
@@ -3280,7 +3280,7 @@
         <v>11</v>
       </c>
       <c r="D5" s="2">
-        <v>24</v>
+        <v>7</v>
       </c>
       <c r="E5" s="2">
         <v>1</v>
@@ -3309,7 +3309,7 @@
         <v>11</v>
       </c>
       <c r="D6" s="2">
-        <v>28</v>
+        <v>8</v>
       </c>
       <c r="E6" s="2">
         <v>2</v>
@@ -3338,7 +3338,7 @@
         <v>11</v>
       </c>
       <c r="D7" s="2">
-        <v>30</v>
+        <v>9</v>
       </c>
       <c r="E7" s="2">
         <v>2</v>
@@ -3367,7 +3367,7 @@
         <v>11</v>
       </c>
       <c r="D8" s="2">
-        <v>34</v>
+        <v>10</v>
       </c>
       <c r="E8" s="2">
         <v>3</v>
@@ -3396,7 +3396,7 @@
         <v>11</v>
       </c>
       <c r="D9" s="2">
-        <v>20</v>
+        <v>6</v>
       </c>
       <c r="E9" s="2">
         <v>1</v>
@@ -3425,7 +3425,7 @@
         <v>11</v>
       </c>
       <c r="D10" s="2">
-        <v>28</v>
+        <v>8</v>
       </c>
       <c r="E10" s="2">
         <v>2</v>
@@ -3454,7 +3454,7 @@
         <v>11</v>
       </c>
       <c r="D11" s="2">
-        <v>36</v>
+        <v>11</v>
       </c>
       <c r="E11" s="2">
         <v>3</v>
@@ -3483,7 +3483,7 @@
         <v>11</v>
       </c>
       <c r="D12" s="2">
-        <v>30</v>
+        <v>8</v>
       </c>
       <c r="E12" s="2">
         <v>2</v>
@@ -3512,7 +3512,7 @@
         <v>11</v>
       </c>
       <c r="D13" s="2">
-        <v>34</v>
+        <v>10</v>
       </c>
       <c r="E13" s="2">
         <v>3</v>
@@ -3541,7 +3541,7 @@
         <v>11</v>
       </c>
       <c r="D14" s="2">
-        <v>26</v>
+        <v>7</v>
       </c>
       <c r="E14" s="2">
         <v>2</v>
@@ -3570,7 +3570,7 @@
         <v>11</v>
       </c>
       <c r="D15" s="2">
-        <v>32</v>
+        <v>10</v>
       </c>
       <c r="E15" s="2">
         <v>3</v>
@@ -3599,7 +3599,7 @@
         <v>11</v>
       </c>
       <c r="D16" s="2">
-        <v>38</v>
+        <v>12</v>
       </c>
       <c r="E16" s="2">
         <v>3</v>

</xml_diff>

<commit_message>
Sync branch updates and ornament rune naming
</commit_message>
<xml_diff>
--- a/spec/Docs/01_Design/CardDesignVersion/物品列表.xlsx
+++ b/spec/Docs/01_Design/CardDesignVersion/物品列表.xlsx
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="500" uniqueCount="269">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="270" uniqueCount="270">
   <si>
     <t>序号</t>
   </si>
@@ -832,6 +832,9 @@
   </si>
   <si>
     <t>刷新目标饰品“每个局内关卡限 1 次”的触发次数，每饰品每关最多刷新 1 次。</t>
+  </si>
+  <si>
+    <t>目标食物本局内丢弃时额外 +2 梦值。</t>
   </si>
 </sst>
 </file>
@@ -2158,8 +2161,8 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:J20"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <dimension ref="A1:J5"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="8.7109375" customWidth="1"/>
@@ -2330,486 +2333,6 @@
       </c>
       <c r="J5" s="3" t="s">
         <v>135</v>
-      </c>
-    </row>
-    <row r="6" spans="1:10">
-      <c r="A6" s="2">
-        <v>5</v>
-      </c>
-      <c r="B6" s="3" t="s">
-        <v>136</v>
-      </c>
-      <c r="C6" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="D6" s="2">
-        <v>6</v>
-      </c>
-      <c r="E6" s="2">
-        <v>2</v>
-      </c>
-      <c r="F6" s="3" t="s">
-        <v>119</v>
-      </c>
-      <c r="G6" s="3" t="s">
-        <v>13</v>
-      </c>
-      <c r="H6" s="3" t="s">
-        <v>137</v>
-      </c>
-      <c r="I6" s="3" t="s">
-        <v>138</v>
-      </c>
-      <c r="J6" s="3" t="s">
-        <v>139</v>
-      </c>
-    </row>
-    <row r="7" spans="1:10">
-      <c r="A7" s="2">
-        <v>6</v>
-      </c>
-      <c r="B7" s="3" t="s">
-        <v>140</v>
-      </c>
-      <c r="C7" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="D7" s="2">
-        <v>5</v>
-      </c>
-      <c r="E7" s="2">
-        <v>1</v>
-      </c>
-      <c r="F7" s="3" t="s">
-        <v>119</v>
-      </c>
-      <c r="G7" s="3" t="s">
-        <v>13</v>
-      </c>
-      <c r="H7" s="3" t="s">
-        <v>141</v>
-      </c>
-      <c r="I7" s="3" t="s">
-        <v>142</v>
-      </c>
-      <c r="J7" s="3" t="s">
-        <v>143</v>
-      </c>
-    </row>
-    <row r="8" spans="1:10">
-      <c r="A8" s="2">
-        <v>7</v>
-      </c>
-      <c r="B8" s="3" t="s">
-        <v>144</v>
-      </c>
-      <c r="C8" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="D8" s="2">
-        <v>3</v>
-      </c>
-      <c r="E8" s="2">
-        <v>1</v>
-      </c>
-      <c r="F8" s="3" t="s">
-        <v>119</v>
-      </c>
-      <c r="G8" s="3" t="s">
-        <v>145</v>
-      </c>
-      <c r="H8" s="3" t="s">
-        <v>146</v>
-      </c>
-      <c r="I8" s="3" t="s">
-        <v>147</v>
-      </c>
-      <c r="J8" s="3" t="s">
-        <v>148</v>
-      </c>
-    </row>
-    <row r="9" spans="1:10">
-      <c r="A9" s="2">
-        <v>8</v>
-      </c>
-      <c r="B9" s="3" t="s">
-        <v>149</v>
-      </c>
-      <c r="C9" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="D9" s="2">
-        <v>7</v>
-      </c>
-      <c r="E9" s="2">
-        <v>2</v>
-      </c>
-      <c r="F9" s="3" t="s">
-        <v>119</v>
-      </c>
-      <c r="G9" s="3" t="s">
-        <v>13</v>
-      </c>
-      <c r="H9" s="3" t="s">
-        <v>150</v>
-      </c>
-      <c r="I9" s="3" t="s">
-        <v>151</v>
-      </c>
-      <c r="J9" s="3" t="s">
-        <v>152</v>
-      </c>
-    </row>
-    <row r="10" spans="1:10">
-      <c r="A10" s="2">
-        <v>9</v>
-      </c>
-      <c r="B10" s="3" t="s">
-        <v>153</v>
-      </c>
-      <c r="C10" s="3" t="s">
-        <v>23</v>
-      </c>
-      <c r="D10" s="2">
-        <v>8</v>
-      </c>
-      <c r="E10" s="2">
-        <v>3</v>
-      </c>
-      <c r="F10" s="3" t="s">
-        <v>119</v>
-      </c>
-      <c r="G10" s="3" t="s">
-        <v>24</v>
-      </c>
-      <c r="H10" s="3" t="s">
-        <v>154</v>
-      </c>
-      <c r="I10" s="3" t="s">
-        <v>155</v>
-      </c>
-      <c r="J10" s="3" t="s">
-        <v>156</v>
-      </c>
-    </row>
-    <row r="11" spans="1:10">
-      <c r="A11" s="2">
-        <v>10</v>
-      </c>
-      <c r="B11" s="3" t="s">
-        <v>157</v>
-      </c>
-      <c r="C11" s="3" t="s">
-        <v>23</v>
-      </c>
-      <c r="D11" s="2">
-        <v>8</v>
-      </c>
-      <c r="E11" s="2">
-        <v>2</v>
-      </c>
-      <c r="F11" s="3" t="s">
-        <v>119</v>
-      </c>
-      <c r="G11" s="3" t="s">
-        <v>40</v>
-      </c>
-      <c r="H11" s="3" t="s">
-        <v>158</v>
-      </c>
-      <c r="I11" s="3" t="s">
-        <v>159</v>
-      </c>
-      <c r="J11" s="3" t="s">
-        <v>160</v>
-      </c>
-    </row>
-    <row r="12" spans="1:10">
-      <c r="A12" s="2">
-        <v>11</v>
-      </c>
-      <c r="B12" s="3" t="s">
-        <v>161</v>
-      </c>
-      <c r="C12" s="3" t="s">
-        <v>44</v>
-      </c>
-      <c r="D12" s="2">
-        <v>12</v>
-      </c>
-      <c r="E12" s="2">
-        <v>5</v>
-      </c>
-      <c r="F12" s="3" t="s">
-        <v>162</v>
-      </c>
-      <c r="G12" s="3" t="s">
-        <v>24</v>
-      </c>
-      <c r="H12" s="3" t="s">
-        <v>163</v>
-      </c>
-      <c r="I12" s="3" t="s">
-        <v>164</v>
-      </c>
-      <c r="J12" s="3" t="s">
-        <v>165</v>
-      </c>
-    </row>
-    <row r="13" spans="1:10">
-      <c r="A13" s="2">
-        <v>12</v>
-      </c>
-      <c r="B13" s="3" t="s">
-        <v>166</v>
-      </c>
-      <c r="C13" s="3" t="s">
-        <v>28</v>
-      </c>
-      <c r="D13" s="2">
-        <v>15</v>
-      </c>
-      <c r="E13" s="2">
-        <v>6</v>
-      </c>
-      <c r="F13" s="3" t="s">
-        <v>162</v>
-      </c>
-      <c r="G13" s="3" t="s">
-        <v>13</v>
-      </c>
-      <c r="H13" s="3" t="s">
-        <v>167</v>
-      </c>
-      <c r="I13" s="3" t="s">
-        <v>168</v>
-      </c>
-      <c r="J13" s="3" t="s">
-        <v>169</v>
-      </c>
-    </row>
-    <row r="14" spans="1:10">
-      <c r="A14" s="2">
-        <v>13</v>
-      </c>
-      <c r="B14" s="3" t="s">
-        <v>170</v>
-      </c>
-      <c r="C14" s="3" t="s">
-        <v>23</v>
-      </c>
-      <c r="D14" s="2">
-        <v>12</v>
-      </c>
-      <c r="E14" s="2">
-        <v>5</v>
-      </c>
-      <c r="F14" s="3" t="s">
-        <v>119</v>
-      </c>
-      <c r="G14" s="3" t="s">
-        <v>40</v>
-      </c>
-      <c r="H14" s="3" t="s">
-        <v>171</v>
-      </c>
-      <c r="I14" s="3" t="s">
-        <v>172</v>
-      </c>
-      <c r="J14" s="3" t="s">
-        <v>173</v>
-      </c>
-    </row>
-    <row r="15" spans="1:10">
-      <c r="A15" s="2">
-        <v>14</v>
-      </c>
-      <c r="B15" s="3" t="s">
-        <v>174</v>
-      </c>
-      <c r="C15" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="D15" s="2">
-        <v>14</v>
-      </c>
-      <c r="E15" s="2">
-        <v>6</v>
-      </c>
-      <c r="F15" s="3" t="s">
-        <v>119</v>
-      </c>
-      <c r="G15" s="3" t="s">
-        <v>13</v>
-      </c>
-      <c r="H15" s="3" t="s">
-        <v>175</v>
-      </c>
-      <c r="I15" s="3" t="s">
-        <v>176</v>
-      </c>
-      <c r="J15" s="3" t="s">
-        <v>177</v>
-      </c>
-    </row>
-    <row r="16" spans="1:10">
-      <c r="A16" s="2">
-        <v>15</v>
-      </c>
-      <c r="B16" s="3" t="s">
-        <v>178</v>
-      </c>
-      <c r="C16" s="3" t="s">
-        <v>28</v>
-      </c>
-      <c r="D16" s="2">
-        <v>18</v>
-      </c>
-      <c r="E16" s="2">
-        <v>7</v>
-      </c>
-      <c r="F16" s="3" t="s">
-        <v>119</v>
-      </c>
-      <c r="G16" s="3" t="s">
-        <v>13</v>
-      </c>
-      <c r="H16" s="3" t="s">
-        <v>179</v>
-      </c>
-      <c r="I16" s="3" t="s">
-        <v>180</v>
-      </c>
-      <c r="J16" s="3" t="s">
-        <v>181</v>
-      </c>
-    </row>
-    <row r="17" spans="1:10">
-      <c r="A17" s="2">
-        <v>16</v>
-      </c>
-      <c r="B17" s="3" t="s">
-        <v>182</v>
-      </c>
-      <c r="C17" s="3" t="s">
-        <v>28</v>
-      </c>
-      <c r="D17" s="2">
-        <v>20</v>
-      </c>
-      <c r="E17" s="2">
-        <v>8</v>
-      </c>
-      <c r="F17" s="3" t="s">
-        <v>162</v>
-      </c>
-      <c r="G17" s="3" t="s">
-        <v>13</v>
-      </c>
-      <c r="H17" s="3" t="s">
-        <v>183</v>
-      </c>
-      <c r="I17" s="3" t="s">
-        <v>184</v>
-      </c>
-      <c r="J17" s="3" t="s">
-        <v>185</v>
-      </c>
-    </row>
-    <row r="18" spans="1:10">
-      <c r="A18" s="2">
-        <v>17</v>
-      </c>
-      <c r="B18" s="3" t="s">
-        <v>186</v>
-      </c>
-      <c r="C18" s="3" t="s">
-        <v>48</v>
-      </c>
-      <c r="D18" s="2">
-        <v>25</v>
-      </c>
-      <c r="E18" s="2">
-        <v>14</v>
-      </c>
-      <c r="F18" s="3" t="s">
-        <v>119</v>
-      </c>
-      <c r="G18" s="3" t="s">
-        <v>13</v>
-      </c>
-      <c r="H18" s="3" t="s">
-        <v>187</v>
-      </c>
-      <c r="I18" s="3" t="s">
-        <v>188</v>
-      </c>
-      <c r="J18" s="3" t="s">
-        <v>189</v>
-      </c>
-    </row>
-    <row r="19" spans="1:10">
-      <c r="A19" s="2">
-        <v>18</v>
-      </c>
-      <c r="B19" s="3" t="s">
-        <v>190</v>
-      </c>
-      <c r="C19" s="3" t="s">
-        <v>109</v>
-      </c>
-      <c r="D19" s="2">
-        <v>30</v>
-      </c>
-      <c r="E19" s="2">
-        <v>16</v>
-      </c>
-      <c r="F19" s="3" t="s">
-        <v>119</v>
-      </c>
-      <c r="G19" s="3" t="s">
-        <v>24</v>
-      </c>
-      <c r="H19" s="3" t="s">
-        <v>191</v>
-      </c>
-      <c r="I19" s="3" t="s">
-        <v>192</v>
-      </c>
-      <c r="J19" s="3" t="s">
-        <v>193</v>
-      </c>
-    </row>
-    <row r="20" spans="1:10">
-      <c r="A20" s="2">
-        <v>19</v>
-      </c>
-      <c r="B20" s="3" t="s">
-        <v>194</v>
-      </c>
-      <c r="C20" s="3" t="s">
-        <v>28</v>
-      </c>
-      <c r="D20" s="2">
-        <v>26</v>
-      </c>
-      <c r="E20" s="2">
-        <v>15</v>
-      </c>
-      <c r="F20" s="3" t="s">
-        <v>119</v>
-      </c>
-      <c r="G20" s="3" t="s">
-        <v>13</v>
-      </c>
-      <c r="H20" s="3" t="s">
-        <v>195</v>
-      </c>
-      <c r="I20" s="3" t="s">
-        <v>196</v>
-      </c>
-      <c r="J20" s="3" t="s">
-        <v>197</v>
       </c>
     </row>
   </sheetData>
@@ -3140,7 +2663,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:I16"/>
+  <dimension ref="A1:I13"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="8.7109375" customWidth="1"/>
@@ -3390,16 +2913,16 @@
         <v>8</v>
       </c>
       <c r="B9" s="3" t="s">
-        <v>246</v>
+        <v>255</v>
       </c>
       <c r="C9" s="3" t="s">
         <v>11</v>
       </c>
       <c r="D9" s="2">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="E9" s="2">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F9" s="3" t="s">
         <v>224</v>
@@ -3408,10 +2931,10 @@
         <v>117</v>
       </c>
       <c r="H9" s="3" t="s">
-        <v>247</v>
+        <v>256</v>
       </c>
       <c r="I9" s="3" t="s">
-        <v>248</v>
+        <v>257</v>
       </c>
     </row>
     <row r="10" spans="1:9">
@@ -3419,28 +2942,28 @@
         <v>9</v>
       </c>
       <c r="B10" s="3" t="s">
-        <v>249</v>
+        <v>258</v>
       </c>
       <c r="C10" s="3" t="s">
         <v>11</v>
       </c>
       <c r="D10" s="2">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="E10" s="2">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F10" s="3" t="s">
-        <v>224</v>
+        <v>243</v>
       </c>
       <c r="G10" s="3" t="s">
         <v>117</v>
       </c>
       <c r="H10" s="3" t="s">
-        <v>250</v>
+        <v>259</v>
       </c>
       <c r="I10" s="3" t="s">
-        <v>251</v>
+        <v>260</v>
       </c>
     </row>
     <row r="11" spans="1:9">
@@ -3448,28 +2971,28 @@
         <v>10</v>
       </c>
       <c r="B11" s="3" t="s">
-        <v>252</v>
+        <v>261</v>
       </c>
       <c r="C11" s="3" t="s">
         <v>11</v>
       </c>
       <c r="D11" s="2">
-        <v>11</v>
+        <v>7</v>
       </c>
       <c r="E11" s="2">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F11" s="3" t="s">
-        <v>243</v>
+        <v>224</v>
       </c>
       <c r="G11" s="3" t="s">
         <v>117</v>
       </c>
       <c r="H11" s="3" t="s">
-        <v>253</v>
+        <v>269</v>
       </c>
       <c r="I11" s="3" t="s">
-        <v>254</v>
+        <v>263</v>
       </c>
     </row>
     <row r="12" spans="1:9">
@@ -3477,28 +3000,28 @@
         <v>11</v>
       </c>
       <c r="B12" s="3" t="s">
-        <v>255</v>
+        <v>264</v>
       </c>
       <c r="C12" s="3" t="s">
         <v>11</v>
       </c>
       <c r="D12" s="2">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="E12" s="2">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F12" s="3" t="s">
-        <v>224</v>
+        <v>243</v>
       </c>
       <c r="G12" s="3" t="s">
         <v>117</v>
       </c>
       <c r="H12" s="3" t="s">
-        <v>256</v>
+        <v>265</v>
       </c>
       <c r="I12" s="3" t="s">
-        <v>257</v>
+        <v>266</v>
       </c>
     </row>
     <row r="13" spans="1:9">
@@ -3506,13 +3029,13 @@
         <v>12</v>
       </c>
       <c r="B13" s="3" t="s">
-        <v>258</v>
+        <v>267</v>
       </c>
       <c r="C13" s="3" t="s">
         <v>11</v>
       </c>
       <c r="D13" s="2">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="E13" s="2">
         <v>3</v>
@@ -3524,96 +3047,9 @@
         <v>117</v>
       </c>
       <c r="H13" s="3" t="s">
-        <v>259</v>
+        <v>268</v>
       </c>
       <c r="I13" s="3" t="s">
-        <v>260</v>
-      </c>
-    </row>
-    <row r="14" spans="1:9">
-      <c r="A14" s="2">
-        <v>13</v>
-      </c>
-      <c r="B14" s="3" t="s">
-        <v>261</v>
-      </c>
-      <c r="C14" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="D14" s="2">
-        <v>7</v>
-      </c>
-      <c r="E14" s="2">
-        <v>2</v>
-      </c>
-      <c r="F14" s="3" t="s">
-        <v>224</v>
-      </c>
-      <c r="G14" s="3" t="s">
-        <v>117</v>
-      </c>
-      <c r="H14" s="3" t="s">
-        <v>262</v>
-      </c>
-      <c r="I14" s="3" t="s">
-        <v>263</v>
-      </c>
-    </row>
-    <row r="15" spans="1:9">
-      <c r="A15" s="2">
-        <v>14</v>
-      </c>
-      <c r="B15" s="3" t="s">
-        <v>264</v>
-      </c>
-      <c r="C15" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="D15" s="2">
-        <v>10</v>
-      </c>
-      <c r="E15" s="2">
-        <v>3</v>
-      </c>
-      <c r="F15" s="3" t="s">
-        <v>243</v>
-      </c>
-      <c r="G15" s="3" t="s">
-        <v>117</v>
-      </c>
-      <c r="H15" s="3" t="s">
-        <v>265</v>
-      </c>
-      <c r="I15" s="3" t="s">
-        <v>266</v>
-      </c>
-    </row>
-    <row r="16" spans="1:9">
-      <c r="A16" s="2">
-        <v>15</v>
-      </c>
-      <c r="B16" s="3" t="s">
-        <v>267</v>
-      </c>
-      <c r="C16" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="D16" s="2">
-        <v>12</v>
-      </c>
-      <c r="E16" s="2">
-        <v>3</v>
-      </c>
-      <c r="F16" s="3" t="s">
-        <v>243</v>
-      </c>
-      <c r="G16" s="3" t="s">
-        <v>117</v>
-      </c>
-      <c r="H16" s="3" t="s">
-        <v>268</v>
-      </c>
-      <c r="I16" s="3" t="s">
         <v>267</v>
       </c>
     </row>

</xml_diff>